<commit_message>
build based on ee206d8
</commit_message>
<xml_diff>
--- a/previews/PR34/examples/results/output_file_CO.xlsx
+++ b/previews/PR34/examples/results/output_file_CO.xlsx
@@ -553,7 +553,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>3.7438533306121826</v>
+        <v>3.0205295085906982</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -600,10 +600,10 @@
         <v>45181.850661596065</v>
       </c>
       <c r="D2">
-        <v>-1.2064931898647628e6</v>
+        <v>-1.2065231898647628e6</v>
       </c>
       <c r="E2">
-        <v>-1.2064931898647628e6</v>
+        <v>-1.2065231898647628e6</v>
       </c>
       <c r="F2">
         <v>3036.930062754793</v>
@@ -878,7 +878,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>-570716.9482471673</v>
+        <v>-570726.9482471673</v>
       </c>
       <c r="C2">
         <v>69355.85492709026</v>
@@ -924,7 +924,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>-229654.1601644049</v>
+        <v>-229664.1601644049</v>
       </c>
       <c r="C3">
         <v>67340.62813169464</v>
@@ -978,7 +978,7 @@
         <v>32</v>
       </c>
       <c r="B4">
-        <v>-451303.9321147784</v>
+        <v>-451313.9321147784</v>
       </c>
       <c r="C4">
         <v>259791.10814409857</v>

</xml_diff>

<commit_message>
build based on 2d7666e
</commit_message>
<xml_diff>
--- a/previews/PR34/examples/results/output_file_CO.xlsx
+++ b/previews/PR34/examples/results/output_file_CO.xlsx
@@ -553,7 +553,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>3.0205295085906982</v>
+        <v>3.6800496578216553</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -600,10 +600,10 @@
         <v>45181.850661596065</v>
       </c>
       <c r="D2">
-        <v>-1.2065231898647628e6</v>
+        <v>-1.2064931898647628e6</v>
       </c>
       <c r="E2">
-        <v>-1.2065231898647628e6</v>
+        <v>-1.2064931898647628e6</v>
       </c>
       <c r="F2">
         <v>3036.930062754793</v>
@@ -878,7 +878,7 @@
         <v>30</v>
       </c>
       <c r="B2">
-        <v>-570726.9482471673</v>
+        <v>-570716.9482471673</v>
       </c>
       <c r="C2">
         <v>69355.85492709026</v>
@@ -924,7 +924,7 @@
         <v>31</v>
       </c>
       <c r="B3">
-        <v>-229664.1601644049</v>
+        <v>-229654.1601644049</v>
       </c>
       <c r="C3">
         <v>67340.62813169464</v>
@@ -978,7 +978,7 @@
         <v>32</v>
       </c>
       <c r="B4">
-        <v>-451313.9321147784</v>
+        <v>-451303.9321147784</v>
       </c>
       <c r="C4">
         <v>259791.10814409857</v>

</xml_diff>